<commit_message>
docs: changed fase to room
</commit_message>
<xml_diff>
--- a/docs/planilha_fases_jogo.xlsx
+++ b/docs/planilha_fases_jogo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ThinkPad\Documents\GitHub\gravity-rooms\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D8D0602-1B85-49EB-BE27-D66627A6D8B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0DDD630-04B1-40F9-9935-3CDDCBC0F591}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,9 +22,6 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="71">
   <si>
-    <t>Nome da fase</t>
-  </si>
-  <si>
     <t>Mecânicas usadas</t>
   </si>
   <si>
@@ -34,9 +31,6 @@
     <t>Tempo de gameplay (s)</t>
   </si>
   <si>
-    <t>fase_01_neon_lab_easy</t>
-  </si>
-  <si>
     <t>movimento + pulo + inverter gravidade</t>
   </si>
   <si>
@@ -46,183 +40,96 @@
     <t>30-45</t>
   </si>
   <si>
-    <t>fase_02_neon_lab_easy</t>
-  </si>
-  <si>
     <t>gravidade + chave simples</t>
   </si>
   <si>
-    <t>fase_03_neon_lab_easy</t>
-  </si>
-  <si>
     <t>sequência de 2 inversões</t>
   </si>
   <si>
-    <t>fase_04_ruins_ancient_easy</t>
-  </si>
-  <si>
     <t>espinhos + posicionamento</t>
   </si>
   <si>
-    <t>fase_05_ruins_ancient_easy</t>
-  </si>
-  <si>
     <t>gravidade para evitar dano</t>
   </si>
   <si>
-    <t>fase_06_ruins_ancient_easy</t>
-  </si>
-  <si>
     <t>timing leve + armadilhas</t>
   </si>
   <si>
-    <t>fase_07_crystal_caves_easy</t>
-  </si>
-  <si>
     <t>guias visuais (cristais)</t>
   </si>
   <si>
-    <t>fase_08_crystal_caves_easy</t>
-  </si>
-  <si>
     <t>caminhos alternativos</t>
   </si>
   <si>
-    <t>fase_09_crystal_caves_easy</t>
-  </si>
-  <si>
     <t>puzzle vertical</t>
   </si>
   <si>
-    <t>fase_10_lava_forge_easy</t>
-  </si>
-  <si>
     <t>lava + timing básico</t>
   </si>
   <si>
-    <t>fase_11_lava_forge_normal</t>
-  </si>
-  <si>
     <t>plataformas móveis + lava</t>
   </si>
   <si>
     <t>45-70</t>
   </si>
   <si>
-    <t>fase_12_lava_forge_normal</t>
-  </si>
-  <si>
     <t>sequência rápida + gravidade</t>
   </si>
   <si>
-    <t>fase_13_sky_ruins_normal</t>
-  </si>
-  <si>
     <t>grandes saltos + gravidade</t>
   </si>
   <si>
-    <t>fase_14_sky_ruins_normal</t>
-  </si>
-  <si>
     <t>rotas alternativas aéreas</t>
   </si>
   <si>
-    <t>fase_15_sky_ruins_normal</t>
-  </si>
-  <si>
     <t>precisão de inversão</t>
   </si>
   <si>
-    <t>fase_16_deep_forest_normal</t>
-  </si>
-  <si>
     <t>exploração + múltiplos caminhos</t>
   </si>
   <si>
-    <t>fase_17_deep_forest_normal</t>
-  </si>
-  <si>
     <t>backtracking + chave</t>
   </si>
   <si>
-    <t>fase_18_deep_forest_normal</t>
-  </si>
-  <si>
     <t>puzzle espacial</t>
   </si>
   <si>
-    <t>fase_19_ice_temple_normal</t>
-  </si>
-  <si>
     <t>superfície escorregadia</t>
   </si>
   <si>
-    <t>fase_20_ice_temple_normal</t>
-  </si>
-  <si>
     <t>inércia + gravidade</t>
   </si>
   <si>
-    <t>fase_21_ice_temple_hard</t>
-  </si>
-  <si>
     <t>precisão extrema + gelo</t>
   </si>
   <si>
     <t>60-90</t>
   </si>
   <si>
-    <t>fase_22_abandoned_station_hard</t>
-  </si>
-  <si>
     <t>zonas de gravidade</t>
   </si>
   <si>
-    <t>fase_23_abandoned_station_hard</t>
-  </si>
-  <si>
     <t>áreas sem gravidade</t>
   </si>
   <si>
-    <t>fase_24_abandoned_station_hard</t>
-  </si>
-  <si>
     <t>transição entre físicas</t>
   </si>
   <si>
-    <t>fase_25_shadow_realm_hard</t>
-  </si>
-  <si>
     <t>plataformas invisíveis</t>
   </si>
   <si>
-    <t>fase_26_shadow_realm_hard</t>
-  </si>
-  <si>
     <t>memorização de rota</t>
   </si>
   <si>
-    <t>fase_27_shadow_realm_hard</t>
-  </si>
-  <si>
     <t>execução sob pressão</t>
   </si>
   <si>
-    <t>fase_28_gravity_core_hard</t>
-  </si>
-  <si>
     <t>combinação de mecânicas</t>
   </si>
   <si>
-    <t>fase_29_gravity_core_hard</t>
-  </si>
-  <si>
     <t>sequência longa</t>
   </si>
   <si>
-    <t>fase_30_gravity_core_hard</t>
-  </si>
-  <si>
     <t>desafio final completo</t>
   </si>
   <si>
@@ -233,6 +140,99 @@
   </si>
   <si>
     <t>Tempo real do jogador</t>
+  </si>
+  <si>
+    <t>Nome da Fase</t>
+  </si>
+  <si>
+    <t>room_01_neon_lab_easy</t>
+  </si>
+  <si>
+    <t>room_02_neon_lab_easy</t>
+  </si>
+  <si>
+    <t>room_03_neon_lab_easy</t>
+  </si>
+  <si>
+    <t>room_04_ruins_ancient_easy</t>
+  </si>
+  <si>
+    <t>room_05_ruins_ancient_easy</t>
+  </si>
+  <si>
+    <t>room_06_ruins_ancient_easy</t>
+  </si>
+  <si>
+    <t>room_07_crystal_caves_easy</t>
+  </si>
+  <si>
+    <t>room_08_crystal_caves_easy</t>
+  </si>
+  <si>
+    <t>room_09_crystal_caves_easy</t>
+  </si>
+  <si>
+    <t>room_10_lava_forge_easy</t>
+  </si>
+  <si>
+    <t>room_11_lava_forge_normal</t>
+  </si>
+  <si>
+    <t>room_12_lava_forge_normal</t>
+  </si>
+  <si>
+    <t>room_13_sky_ruins_normal</t>
+  </si>
+  <si>
+    <t>room_14_sky_ruins_normal</t>
+  </si>
+  <si>
+    <t>room_15_sky_ruins_normal</t>
+  </si>
+  <si>
+    <t>room_16_deep_forest_normal</t>
+  </si>
+  <si>
+    <t>room_17_deep_forest_normal</t>
+  </si>
+  <si>
+    <t>room_18_deep_forest_normal</t>
+  </si>
+  <si>
+    <t>room_19_ice_temple_normal</t>
+  </si>
+  <si>
+    <t>room_20_ice_temple_normal</t>
+  </si>
+  <si>
+    <t>room_21_ice_temple_hard</t>
+  </si>
+  <si>
+    <t>room_22_abandoned_station_hard</t>
+  </si>
+  <si>
+    <t>room_23_abandoned_station_hard</t>
+  </si>
+  <si>
+    <t>room_24_abandoned_station_hard</t>
+  </si>
+  <si>
+    <t>room_25_shadow_realm_hard</t>
+  </si>
+  <si>
+    <t>room_26_shadow_realm_hard</t>
+  </si>
+  <si>
+    <t>room_27_shadow_realm_hard</t>
+  </si>
+  <si>
+    <t>room_28_gravity_core_hard</t>
+  </si>
+  <si>
+    <t>room_29_gravity_core_hard</t>
+  </si>
+  <si>
+    <t>room_30_gravity_core_hard</t>
   </si>
 </sst>
 </file>
@@ -586,445 +586,445 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
-        <v>3</v>
-      </c>
       <c r="E1" t="s">
-        <v>68</v>
+        <v>37</v>
       </c>
       <c r="F1" t="s">
-        <v>69</v>
+        <v>38</v>
       </c>
       <c r="G1" t="s">
-        <v>70</v>
+        <v>39</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>4</v>
+        <v>41</v>
       </c>
       <c r="B2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D2" t="s">
         <v>5</v>
-      </c>
-      <c r="C2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D2" t="s">
-        <v>7</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>8</v>
+        <v>42</v>
       </c>
       <c r="B3" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="C3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D3" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>10</v>
+        <v>43</v>
       </c>
       <c r="B4" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="C4" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D4" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>12</v>
+        <v>44</v>
       </c>
       <c r="B5" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="C5" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D5" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>14</v>
+        <v>45</v>
       </c>
       <c r="B6" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="C6" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D6" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>16</v>
+        <v>46</v>
       </c>
       <c r="B7" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="C7" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D7" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>18</v>
+        <v>47</v>
       </c>
       <c r="B8" t="s">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="C8" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D8" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>20</v>
+        <v>48</v>
       </c>
       <c r="B9" t="s">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="C9" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D9" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>22</v>
+        <v>49</v>
       </c>
       <c r="B10" t="s">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="C10" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D10" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>24</v>
+        <v>50</v>
       </c>
       <c r="B11" t="s">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="C11" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D11" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>26</v>
+        <v>51</v>
       </c>
       <c r="B12" t="s">
-        <v>27</v>
+        <v>15</v>
       </c>
       <c r="C12" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D12" t="s">
-        <v>28</v>
+        <v>16</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>29</v>
+        <v>52</v>
       </c>
       <c r="B13" t="s">
-        <v>30</v>
+        <v>17</v>
       </c>
       <c r="C13" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D13" t="s">
-        <v>28</v>
+        <v>16</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>31</v>
+        <v>53</v>
       </c>
       <c r="B14" t="s">
-        <v>32</v>
+        <v>18</v>
       </c>
       <c r="C14" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D14" t="s">
-        <v>28</v>
+        <v>16</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>33</v>
+        <v>54</v>
       </c>
       <c r="B15" t="s">
-        <v>34</v>
+        <v>19</v>
       </c>
       <c r="C15" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D15" t="s">
-        <v>28</v>
+        <v>16</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>35</v>
+        <v>55</v>
       </c>
       <c r="B16" t="s">
-        <v>36</v>
+        <v>20</v>
       </c>
       <c r="C16" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D16" t="s">
-        <v>28</v>
+        <v>16</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>37</v>
+        <v>56</v>
       </c>
       <c r="B17" t="s">
-        <v>38</v>
+        <v>21</v>
       </c>
       <c r="C17" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D17" t="s">
-        <v>28</v>
+        <v>16</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>39</v>
+        <v>57</v>
       </c>
       <c r="B18" t="s">
-        <v>40</v>
+        <v>22</v>
       </c>
       <c r="C18" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D18" t="s">
-        <v>28</v>
+        <v>16</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>41</v>
+        <v>58</v>
       </c>
       <c r="B19" t="s">
-        <v>42</v>
+        <v>23</v>
       </c>
       <c r="C19" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D19" t="s">
-        <v>28</v>
+        <v>16</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>43</v>
+        <v>59</v>
       </c>
       <c r="B20" t="s">
-        <v>44</v>
+        <v>24</v>
       </c>
       <c r="C20" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D20" t="s">
-        <v>28</v>
+        <v>16</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>45</v>
+        <v>60</v>
       </c>
       <c r="B21" t="s">
-        <v>46</v>
+        <v>25</v>
       </c>
       <c r="C21" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D21" t="s">
-        <v>28</v>
+        <v>16</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>47</v>
+        <v>61</v>
       </c>
       <c r="B22" t="s">
-        <v>48</v>
+        <v>26</v>
       </c>
       <c r="C22" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D22" t="s">
-        <v>49</v>
+        <v>27</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>50</v>
+        <v>62</v>
       </c>
       <c r="B23" t="s">
-        <v>51</v>
+        <v>28</v>
       </c>
       <c r="C23" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D23" t="s">
-        <v>49</v>
+        <v>27</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>52</v>
+        <v>63</v>
       </c>
       <c r="B24" t="s">
-        <v>53</v>
+        <v>29</v>
       </c>
       <c r="C24" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D24" t="s">
-        <v>49</v>
+        <v>27</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>54</v>
+        <v>64</v>
       </c>
       <c r="B25" t="s">
-        <v>55</v>
+        <v>30</v>
       </c>
       <c r="C25" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D25" t="s">
-        <v>49</v>
+        <v>27</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>56</v>
+        <v>65</v>
       </c>
       <c r="B26" t="s">
-        <v>57</v>
+        <v>31</v>
       </c>
       <c r="C26" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D26" t="s">
-        <v>49</v>
+        <v>27</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>58</v>
+        <v>66</v>
       </c>
       <c r="B27" t="s">
-        <v>59</v>
+        <v>32</v>
       </c>
       <c r="C27" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D27" t="s">
-        <v>49</v>
+        <v>27</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>60</v>
+        <v>67</v>
       </c>
       <c r="B28" t="s">
-        <v>61</v>
+        <v>33</v>
       </c>
       <c r="C28" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D28" t="s">
-        <v>49</v>
+        <v>27</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="B29" t="s">
-        <v>63</v>
+        <v>34</v>
       </c>
       <c r="C29" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D29" t="s">
-        <v>49</v>
+        <v>27</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="B30" t="s">
-        <v>65</v>
+        <v>35</v>
       </c>
       <c r="C30" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D30" t="s">
-        <v>49</v>
+        <v>27</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="B31" t="s">
-        <v>67</v>
+        <v>36</v>
       </c>
       <c r="C31" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D31" t="s">
-        <v>49</v>
+        <v>27</v>
       </c>
     </row>
   </sheetData>

</xml_diff>